<commit_message>
#4 eSpark and Client BOM Added
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Board-v1.0/BOM/eSpark-BOM-Main-Board-v1.0.xlsx
+++ b/Design-Files/Main-Board-v1.0/BOM/eSpark-BOM-Main-Board-v1.0.xlsx
@@ -12,14 +12,14 @@
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="452">
   <si>
     <t>Component list</t>
   </si>
@@ -1182,9 +1182,6 @@
     <t>C94361</t>
   </si>
   <si>
-    <t>C2678726</t>
-  </si>
-  <si>
     <t>C2149207</t>
   </si>
   <si>
@@ -1357,6 +1354,27 @@
   </si>
   <si>
     <t>C17477</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Polymer lithium battery, 906090 mobile power charging treasure</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>Chipsmall</t>
+  </si>
+  <si>
+    <t>0805W8F0000T5E</t>
   </si>
 </sst>
 </file>
@@ -1851,7 +1869,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2000,6 +2018,51 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2032,51 +2095,14 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2420,7 +2446,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S87"/>
+  <dimension ref="A1:S89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -2436,7 +2462,7 @@
     <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" customWidth="1"/>
     <col min="16" max="16" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
@@ -2454,15 +2480,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="57"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="72"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1">
       <c r="A2" s="1"/>
@@ -2473,7 +2499,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="52" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -2498,7 +2524,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="53" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -2512,7 +2538,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="58"/>
+      <c r="S3" s="73"/>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="1"/>
@@ -2523,7 +2549,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="53" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -2537,7 +2563,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="59"/>
+      <c r="S4" s="74"/>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="1"/>
@@ -2562,7 +2588,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="59"/>
+      <c r="S5" s="74"/>
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="1"/>
@@ -2583,7 +2609,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="59"/>
+      <c r="S6" s="74"/>
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="1"/>
@@ -2604,7 +2630,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="59"/>
+      <c r="S7" s="74"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1">
       <c r="A8" s="1"/>
@@ -2625,63 +2651,63 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="59"/>
+      <c r="S8" s="74"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="66" t="s">
+      <c r="B9" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="66" t="s">
+      <c r="C9" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="66" t="s">
+      <c r="D9" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="66" t="s">
+      <c r="E9" s="56" t="s">
         <v>105</v>
       </c>
-      <c r="F9" s="66" t="s">
+      <c r="F9" s="56" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="66" t="s">
+      <c r="G9" s="56" t="s">
         <v>222</v>
       </c>
-      <c r="H9" s="66" t="s">
+      <c r="H9" s="56" t="s">
         <v>287</v>
       </c>
-      <c r="I9" s="66" t="s">
+      <c r="I9" s="56" t="s">
+        <v>426</v>
+      </c>
+      <c r="J9" s="56" t="s">
+        <v>319</v>
+      </c>
+      <c r="K9" s="56" t="s">
         <v>427</v>
       </c>
-      <c r="J9" s="66" t="s">
-        <v>319</v>
-      </c>
-      <c r="K9" s="66" t="s">
+      <c r="L9" s="56" t="s">
+        <v>425</v>
+      </c>
+      <c r="M9" s="56" t="s">
         <v>428</v>
       </c>
-      <c r="L9" s="66" t="s">
-        <v>426</v>
-      </c>
-      <c r="M9" s="66" t="s">
+      <c r="N9" s="56" t="s">
         <v>429</v>
       </c>
-      <c r="N9" s="66" t="s">
+      <c r="O9" s="56" t="s">
         <v>430</v>
       </c>
-      <c r="O9" s="66" t="s">
+      <c r="P9" s="56" t="s">
         <v>431</v>
       </c>
-      <c r="P9" s="66" t="s">
+      <c r="Q9" s="56" t="s">
         <v>432</v>
       </c>
-      <c r="Q9" s="66" t="s">
+      <c r="R9" s="56" t="s">
         <v>433</v>
       </c>
-      <c r="R9" s="66" t="s">
+      <c r="S9" s="56" t="s">
         <v>434</v>
-      </c>
-      <c r="S9" s="66" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="24">
@@ -2690,7 +2716,7 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="67" t="s">
+      <c r="C10" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="36" t="s">
@@ -2709,13 +2735,13 @@
         <v>288</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J10" s="36" t="s">
         <v>320</v>
       </c>
       <c r="K10" s="36" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L10" s="36">
         <v>15</v>
@@ -2727,8 +2753,8 @@
       <c r="N10" s="36">
         <v>80</v>
       </c>
-      <c r="O10" s="69" t="s">
-        <v>441</v>
+      <c r="O10" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P10" s="37">
         <v>0.1137</v>
@@ -2743,10 +2769,10 @@
     <row r="11" spans="1:19">
       <c r="A11" s="1"/>
       <c r="B11" s="46">
-        <f t="shared" ref="B11:B85" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B86" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="68" t="s">
+      <c r="C11" s="58" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="50" t="s">
@@ -2765,13 +2791,13 @@
         <v>288</v>
       </c>
       <c r="I11" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J11" s="50" t="s">
         <v>321</v>
       </c>
       <c r="K11" s="50" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="L11" s="50">
         <v>1</v>
@@ -2783,15 +2809,15 @@
       <c r="N11" s="50">
         <v>50</v>
       </c>
-      <c r="O11" s="70" t="s">
-        <v>441</v>
+      <c r="O11" s="60" t="s">
+        <v>440</v>
       </c>
       <c r="P11" s="51">
-        <v>1.46E-2</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="Q11" s="51">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
-        <v>0.73</v>
+        <v>0.85000000000000009</v>
       </c>
       <c r="R11" s="50"/>
       <c r="S11" s="50"/>
@@ -2802,7 +2828,7 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="67" t="s">
+      <c r="C12" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="36" t="s">
@@ -2821,13 +2847,13 @@
         <v>289</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J12" s="36" t="s">
         <v>322</v>
       </c>
       <c r="K12" s="36" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L12" s="36">
         <v>5</v>
@@ -2839,8 +2865,8 @@
       <c r="N12" s="36">
         <v>30</v>
       </c>
-      <c r="O12" s="69" t="s">
-        <v>441</v>
+      <c r="O12" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P12" s="37">
         <v>5.8500000000000003E-2</v>
@@ -2858,11 +2884,11 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="67" t="s">
+      <c r="C13" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="50" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E13" s="50" t="s">
         <v>109</v>
@@ -2877,13 +2903,13 @@
         <v>288</v>
       </c>
       <c r="I13" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J13" s="50" t="s">
         <v>323</v>
       </c>
       <c r="K13" s="50" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="L13" s="50">
         <v>39</v>
@@ -2895,8 +2921,8 @@
       <c r="N13" s="50">
         <v>200</v>
       </c>
-      <c r="O13" s="70" t="s">
-        <v>441</v>
+      <c r="O13" s="60" t="s">
+        <v>440</v>
       </c>
       <c r="P13" s="51">
         <v>1.1000000000000001E-3</v>
@@ -2914,7 +2940,7 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="67" t="s">
+      <c r="C14" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D14" s="36" t="s">
@@ -2933,13 +2959,13 @@
         <v>288</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J14" s="36" t="s">
         <v>324</v>
       </c>
       <c r="K14" s="36" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L14" s="36">
         <v>1</v>
@@ -2951,8 +2977,8 @@
       <c r="N14" s="36">
         <v>20</v>
       </c>
-      <c r="O14" s="71" t="s">
-        <v>441</v>
+      <c r="O14" s="83" t="s">
+        <v>440</v>
       </c>
       <c r="P14" s="37">
         <v>3.39E-2</v>
@@ -2970,7 +2996,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="67" t="s">
+      <c r="C15" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="50" t="s">
@@ -2989,13 +3015,13 @@
         <v>290</v>
       </c>
       <c r="I15" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J15" s="50" t="s">
         <v>325</v>
       </c>
       <c r="K15" s="50" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="L15" s="50">
         <v>2</v>
@@ -3007,8 +3033,8 @@
       <c r="N15" s="50">
         <v>11</v>
       </c>
-      <c r="O15" s="70" t="s">
-        <v>441</v>
+      <c r="O15" s="60" t="s">
+        <v>440</v>
       </c>
       <c r="P15" s="51">
         <v>0.9244</v>
@@ -3026,7 +3052,7 @@
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="67" t="s">
+      <c r="C16" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="36" t="s">
@@ -3045,13 +3071,13 @@
         <v>288</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J16" s="36" t="s">
         <v>326</v>
       </c>
       <c r="K16" s="36" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="L16" s="36">
         <v>1</v>
@@ -3063,8 +3089,8 @@
       <c r="N16" s="36">
         <v>50</v>
       </c>
-      <c r="O16" s="69" t="s">
-        <v>441</v>
+      <c r="O16" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P16" s="37">
         <v>1.72E-2</v>
@@ -3082,7 +3108,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="67" t="s">
+      <c r="C17" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="50" t="s">
@@ -3101,13 +3127,13 @@
         <v>288</v>
       </c>
       <c r="I17" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J17" s="50" t="s">
         <v>327</v>
       </c>
       <c r="K17" s="50" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L17" s="50">
         <v>2</v>
@@ -3119,8 +3145,8 @@
       <c r="N17" s="50">
         <v>100</v>
       </c>
-      <c r="O17" s="70" t="s">
-        <v>441</v>
+      <c r="O17" s="60" t="s">
+        <v>440</v>
       </c>
       <c r="P17" s="51">
         <v>2.8E-3</v>
@@ -3138,7 +3164,7 @@
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="67" t="s">
+      <c r="C18" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="36" t="s">
@@ -3157,13 +3183,13 @@
         <v>288</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J18" s="36" t="s">
         <v>328</v>
       </c>
       <c r="K18" s="36" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="L18" s="36">
         <v>13</v>
@@ -3175,8 +3201,8 @@
       <c r="N18" s="36">
         <v>100</v>
       </c>
-      <c r="O18" s="69" t="s">
-        <v>441</v>
+      <c r="O18" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P18" s="37">
         <v>7.9000000000000008E-3</v>
@@ -3194,7 +3220,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="68" t="s">
+      <c r="C19" s="58" t="s">
         <v>9</v>
       </c>
       <c r="D19" s="50" t="s">
@@ -3212,12 +3238,14 @@
       <c r="H19" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I19" s="50"/>
+      <c r="I19" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J19" s="50" t="s">
         <v>329</v>
       </c>
       <c r="K19" s="50" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L19" s="50">
         <v>4</v>
@@ -3229,8 +3257,8 @@
       <c r="N19" s="50">
         <v>100</v>
       </c>
-      <c r="O19" s="69" t="s">
-        <v>441</v>
+      <c r="O19" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P19" s="51">
         <v>3.0999999999999999E-3</v>
@@ -3248,7 +3276,7 @@
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="67" t="s">
+      <c r="C20" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D20" s="36" t="s">
@@ -3258,7 +3286,7 @@
         <v>116</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G20" s="36" t="s">
         <v>187</v>
@@ -3266,12 +3294,14 @@
       <c r="H20" s="36" t="s">
         <v>291</v>
       </c>
-      <c r="I20" s="36"/>
+      <c r="I20" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J20" s="36" t="s">
         <v>330</v>
       </c>
       <c r="K20" s="36" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="L20" s="36">
         <v>4</v>
@@ -3283,8 +3313,8 @@
       <c r="N20" s="36">
         <v>30</v>
       </c>
-      <c r="O20" s="69" t="s">
-        <v>441</v>
+      <c r="O20" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P20" s="37">
         <v>5.8799999999999998E-2</v>
@@ -3302,7 +3332,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="68" t="s">
+      <c r="C21" s="58" t="s">
         <v>9</v>
       </c>
       <c r="D21" s="50" t="s">
@@ -3320,12 +3350,14 @@
       <c r="H21" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I21" s="50"/>
+      <c r="I21" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J21" s="50" t="s">
         <v>331</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="L21" s="50">
         <v>2</v>
@@ -3337,8 +3369,8 @@
       <c r="N21" s="50">
         <v>100</v>
       </c>
-      <c r="O21" s="69" t="s">
-        <v>441</v>
+      <c r="O21" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P21" s="51">
         <v>4.0000000000000001E-3</v>
@@ -3356,7 +3388,7 @@
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="67" t="s">
+      <c r="C22" s="57" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="36" t="s">
@@ -3374,12 +3406,14 @@
       <c r="H22" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I22" s="36"/>
+      <c r="I22" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J22" s="36" t="s">
         <v>332</v>
       </c>
       <c r="K22" s="36" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="L22" s="36">
         <v>2</v>
@@ -3391,8 +3425,8 @@
       <c r="N22" s="36">
         <v>50</v>
       </c>
-      <c r="O22" s="69" t="s">
-        <v>441</v>
+      <c r="O22" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P22" s="37">
         <v>1.0699999999999999E-2</v>
@@ -3410,7 +3444,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="68" t="s">
+      <c r="C23" s="58" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="50" t="s">
@@ -3428,12 +3462,14 @@
       <c r="H23" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I23" s="50"/>
+      <c r="I23" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J23" s="50" t="s">
         <v>333</v>
       </c>
       <c r="K23" s="50" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="L23" s="50">
         <v>4</v>
@@ -3445,8 +3481,8 @@
       <c r="N23" s="50">
         <v>100</v>
       </c>
-      <c r="O23" s="69" t="s">
-        <v>441</v>
+      <c r="O23" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P23" s="51">
         <v>3.8999999999999998E-3</v>
@@ -3464,7 +3500,7 @@
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="68" t="s">
+      <c r="C24" s="58" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="36" t="s">
@@ -3482,12 +3518,14 @@
       <c r="H24" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I24" s="36"/>
+      <c r="I24" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J24" s="36" t="s">
         <v>334</v>
       </c>
       <c r="K24" s="36" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="L24" s="36">
         <v>1</v>
@@ -3499,8 +3537,8 @@
       <c r="N24" s="36">
         <v>100</v>
       </c>
-      <c r="O24" s="69" t="s">
-        <v>441</v>
+      <c r="O24" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P24" s="37">
         <v>7.4000000000000003E-3</v>
@@ -3518,7 +3556,7 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="67" t="s">
+      <c r="C25" s="57" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="50" t="s">
@@ -3536,12 +3574,14 @@
       <c r="H25" s="50" t="s">
         <v>292</v>
       </c>
-      <c r="I25" s="50"/>
+      <c r="I25" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J25" s="50" t="s">
         <v>335</v>
       </c>
       <c r="K25" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L25" s="50">
         <v>1</v>
@@ -3553,8 +3593,8 @@
       <c r="N25" s="50">
         <v>50</v>
       </c>
-      <c r="O25" s="69" t="s">
-        <v>441</v>
+      <c r="O25" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P25" s="51">
         <v>1.55E-2</v>
@@ -3572,7 +3612,7 @@
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="67" t="s">
+      <c r="C26" s="57" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="36" t="s">
@@ -3590,12 +3630,14 @@
       <c r="H26" s="36" t="s">
         <v>293</v>
       </c>
-      <c r="I26" s="36"/>
+      <c r="I26" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J26" s="36" t="s">
         <v>336</v>
       </c>
       <c r="K26" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L26" s="36">
         <v>1</v>
@@ -3607,8 +3649,8 @@
       <c r="N26" s="36">
         <v>20</v>
       </c>
-      <c r="O26" s="69" t="s">
-        <v>441</v>
+      <c r="O26" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P26" s="37">
         <v>2.3599999999999999E-2</v>
@@ -3626,7 +3668,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="68" t="s">
+      <c r="C27" s="58" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="50" t="s">
@@ -3644,12 +3686,14 @@
       <c r="H27" s="50" t="s">
         <v>294</v>
       </c>
-      <c r="I27" s="50"/>
+      <c r="I27" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J27" s="50" t="s">
         <v>337</v>
       </c>
       <c r="K27" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L27" s="50">
         <v>2</v>
@@ -3661,8 +3705,8 @@
       <c r="N27" s="50">
         <v>20</v>
       </c>
-      <c r="O27" s="69" t="s">
-        <v>441</v>
+      <c r="O27" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P27" s="51">
         <v>2.3099999999999999E-2</v>
@@ -3680,7 +3724,7 @@
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="67" t="s">
+      <c r="C28" s="57" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="36" t="s">
@@ -3698,12 +3742,14 @@
       <c r="H28" s="36" t="s">
         <v>295</v>
       </c>
-      <c r="I28" s="36"/>
+      <c r="I28" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J28" s="36" t="s">
         <v>338</v>
       </c>
       <c r="K28" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L28" s="36">
         <v>7</v>
@@ -3715,8 +3761,8 @@
       <c r="N28" s="36">
         <v>50</v>
       </c>
-      <c r="O28" s="69" t="s">
-        <v>441</v>
+      <c r="O28" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P28" s="37">
         <v>8.8999999999999999E-3</v>
@@ -3734,7 +3780,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="68" t="s">
+      <c r="C29" s="58" t="s">
         <v>11</v>
       </c>
       <c r="D29" s="50" t="s">
@@ -3752,12 +3798,14 @@
       <c r="H29" s="50" t="s">
         <v>296</v>
       </c>
-      <c r="I29" s="50"/>
+      <c r="I29" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J29" s="50" t="s">
         <v>339</v>
       </c>
       <c r="K29" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L29" s="50">
         <v>9</v>
@@ -3769,8 +3817,8 @@
       <c r="N29" s="50">
         <v>50</v>
       </c>
-      <c r="O29" s="69" t="s">
-        <v>441</v>
+      <c r="O29" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P29" s="51">
         <v>5.96E-2</v>
@@ -3788,7 +3836,7 @@
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="67" t="s">
+      <c r="C30" s="57" t="s">
         <v>11</v>
       </c>
       <c r="D30" s="36" t="s">
@@ -3806,12 +3854,14 @@
       <c r="H30" s="36" t="s">
         <v>296</v>
       </c>
-      <c r="I30" s="36"/>
+      <c r="I30" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J30" s="36" t="s">
         <v>340</v>
       </c>
       <c r="K30" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L30" s="36">
         <v>1</v>
@@ -3823,8 +3873,8 @@
       <c r="N30" s="36">
         <v>10</v>
       </c>
-      <c r="O30" s="69" t="s">
-        <v>441</v>
+      <c r="O30" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P30" s="37">
         <v>0.21029999999999999</v>
@@ -3842,7 +3892,7 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="68" t="s">
+      <c r="C31" s="58" t="s">
         <v>12</v>
       </c>
       <c r="D31" s="50" t="s">
@@ -3852,7 +3902,7 @@
         <v>127</v>
       </c>
       <c r="F31" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G31" s="50" t="s">
         <v>195</v>
@@ -3860,12 +3910,14 @@
       <c r="H31" s="50" t="s">
         <v>297</v>
       </c>
-      <c r="I31" s="50"/>
+      <c r="I31" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J31" s="50" t="s">
         <v>341</v>
       </c>
       <c r="K31" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L31" s="50">
         <v>1</v>
@@ -3877,8 +3929,8 @@
       <c r="N31" s="50">
         <v>10</v>
       </c>
-      <c r="O31" s="69" t="s">
-        <v>441</v>
+      <c r="O31" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P31" s="51">
         <v>4.8899999999999999E-2</v>
@@ -3896,7 +3948,7 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="67" t="s">
+      <c r="C32" s="57" t="s">
         <v>13</v>
       </c>
       <c r="D32" s="36" t="s">
@@ -3906,7 +3958,7 @@
         <v>128</v>
       </c>
       <c r="F32" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G32" s="36" t="s">
         <v>196</v>
@@ -3914,12 +3966,14 @@
       <c r="H32" s="36" t="s">
         <v>298</v>
       </c>
-      <c r="I32" s="36"/>
+      <c r="I32" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J32" s="36" t="s">
         <v>342</v>
       </c>
       <c r="K32" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L32" s="36">
         <v>3</v>
@@ -3931,8 +3985,8 @@
       <c r="N32" s="36">
         <v>20</v>
       </c>
-      <c r="O32" s="69" t="s">
-        <v>441</v>
+      <c r="O32" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P32" s="37">
         <v>4.4299999999999999E-2</v>
@@ -3950,7 +4004,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="68" t="s">
+      <c r="C33" s="58" t="s">
         <v>14</v>
       </c>
       <c r="D33" s="50" t="s">
@@ -3960,7 +4014,7 @@
         <v>129</v>
       </c>
       <c r="F33" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G33" s="50" t="s">
         <v>243</v>
@@ -3968,12 +4022,14 @@
       <c r="H33" s="50" t="s">
         <v>299</v>
       </c>
-      <c r="I33" s="50"/>
+      <c r="I33" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J33" s="50" t="s">
         <v>243</v>
       </c>
       <c r="K33" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L33" s="50">
         <v>1</v>
@@ -3985,8 +4041,8 @@
       <c r="N33" s="50">
         <v>12</v>
       </c>
-      <c r="O33" s="69" t="s">
-        <v>441</v>
+      <c r="O33" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P33" s="51">
         <v>6.8000000000000005E-2</v>
@@ -4004,7 +4060,7 @@
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="67" t="s">
+      <c r="C34" s="57" t="s">
         <v>15</v>
       </c>
       <c r="D34" s="36" t="s">
@@ -4014,7 +4070,7 @@
         <v>130</v>
       </c>
       <c r="F34" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G34" s="36" t="s">
         <v>244</v>
@@ -4022,12 +4078,14 @@
       <c r="H34" s="36" t="s">
         <v>297</v>
       </c>
-      <c r="I34" s="36"/>
+      <c r="I34" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J34" s="36" t="s">
         <v>343</v>
       </c>
       <c r="K34" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L34" s="36">
         <v>1</v>
@@ -4039,8 +4097,8 @@
       <c r="N34" s="36">
         <v>20</v>
       </c>
-      <c r="O34" s="69" t="s">
-        <v>441</v>
+      <c r="O34" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P34" s="37">
         <v>3.0200000000000001E-2</v>
@@ -4058,7 +4116,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="68" t="s">
+      <c r="C35" s="58" t="s">
         <v>14</v>
       </c>
       <c r="D35" s="50" t="s">
@@ -4068,7 +4126,7 @@
         <v>131</v>
       </c>
       <c r="F35" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G35" s="50" t="s">
         <v>245</v>
@@ -4076,12 +4134,14 @@
       <c r="H35" s="50" t="s">
         <v>300</v>
       </c>
-      <c r="I35" s="50"/>
+      <c r="I35" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J35" s="50" t="s">
         <v>344</v>
       </c>
       <c r="K35" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L35" s="50">
         <v>1</v>
@@ -4093,8 +4153,8 @@
       <c r="N35" s="50">
         <v>10</v>
       </c>
-      <c r="O35" s="69" t="s">
-        <v>441</v>
+      <c r="O35" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P35" s="51">
         <v>0.3327</v>
@@ -4112,7 +4172,7 @@
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="67" t="s">
+      <c r="C36" s="57" t="s">
         <v>16</v>
       </c>
       <c r="D36" s="36" t="s">
@@ -4122,7 +4182,7 @@
         <v>132</v>
       </c>
       <c r="F36" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G36" s="36" t="s">
         <v>197</v>
@@ -4130,12 +4190,14 @@
       <c r="H36" s="36" t="s">
         <v>301</v>
       </c>
-      <c r="I36" s="36"/>
+      <c r="I36" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J36" s="36" t="s">
         <v>345</v>
       </c>
       <c r="K36" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L36" s="36">
         <v>1</v>
@@ -4147,8 +4209,8 @@
       <c r="N36" s="36">
         <v>6</v>
       </c>
-      <c r="O36" s="69" t="s">
-        <v>441</v>
+      <c r="O36" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P36" s="37">
         <v>1.8726</v>
@@ -4166,7 +4228,7 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="68" t="s">
+      <c r="C37" s="58" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="50" t="s">
@@ -4176,7 +4238,7 @@
         <v>133</v>
       </c>
       <c r="F37" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G37" s="50" t="s">
         <v>198</v>
@@ -4184,12 +4246,14 @@
       <c r="H37" s="50" t="s">
         <v>300</v>
       </c>
-      <c r="I37" s="50"/>
+      <c r="I37" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J37" s="50" t="s">
         <v>346</v>
       </c>
       <c r="K37" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L37" s="50">
         <v>3</v>
@@ -4201,8 +4265,8 @@
       <c r="N37" s="50">
         <v>20</v>
       </c>
-      <c r="O37" s="69" t="s">
-        <v>441</v>
+      <c r="O37" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P37" s="51">
         <v>0.115</v>
@@ -4220,7 +4284,7 @@
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="67" t="s">
+      <c r="C38" s="57" t="s">
         <v>18</v>
       </c>
       <c r="D38" s="36" t="s">
@@ -4230,7 +4294,7 @@
         <v>134</v>
       </c>
       <c r="F38" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G38" s="36" t="s">
         <v>199</v>
@@ -4238,12 +4302,14 @@
       <c r="H38" s="36" t="s">
         <v>302</v>
       </c>
-      <c r="I38" s="36"/>
+      <c r="I38" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J38" s="36" t="s">
         <v>347</v>
       </c>
       <c r="K38" s="36" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="L38" s="36">
         <v>3</v>
@@ -4255,8 +4321,8 @@
       <c r="N38" s="36">
         <v>16</v>
       </c>
-      <c r="O38" s="69" t="s">
-        <v>441</v>
+      <c r="O38" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P38" s="37">
         <v>7.17E-2</v>
@@ -4274,7 +4340,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="58" t="s">
         <v>18</v>
       </c>
       <c r="D39" s="50" t="s">
@@ -4284,7 +4350,7 @@
         <v>135</v>
       </c>
       <c r="F39" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G39" s="50" t="s">
         <v>200</v>
@@ -4292,12 +4358,14 @@
       <c r="H39" s="50" t="s">
         <v>303</v>
       </c>
-      <c r="I39" s="50"/>
+      <c r="I39" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J39" s="50" t="s">
         <v>348</v>
       </c>
       <c r="K39" s="50" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="L39" s="50">
         <v>4</v>
@@ -4309,8 +4377,8 @@
       <c r="N39" s="50">
         <v>25</v>
       </c>
-      <c r="O39" s="69" t="s">
-        <v>441</v>
+      <c r="O39" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P39" s="51">
         <v>0.31559999999999999</v>
@@ -4328,7 +4396,7 @@
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
-      <c r="C40" s="67" t="s">
+      <c r="C40" s="57" t="s">
         <v>19</v>
       </c>
       <c r="D40" s="36" t="s">
@@ -4346,12 +4414,14 @@
       <c r="H40" s="36" t="s">
         <v>304</v>
       </c>
-      <c r="I40" s="36"/>
+      <c r="I40" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J40" s="36" t="s">
         <v>349</v>
       </c>
       <c r="K40" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L40" s="36">
         <v>2</v>
@@ -4363,8 +4433,8 @@
       <c r="N40" s="36">
         <v>20</v>
       </c>
-      <c r="O40" s="69" t="s">
-        <v>441</v>
+      <c r="O40" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P40" s="37">
         <v>2.0799999999999999E-2</v>
@@ -4382,7 +4452,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="68" t="s">
+      <c r="C41" s="58" t="s">
         <v>19</v>
       </c>
       <c r="D41" s="50" t="s">
@@ -4400,12 +4470,14 @@
       <c r="H41" s="50" t="s">
         <v>304</v>
       </c>
-      <c r="I41" s="50"/>
+      <c r="I41" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J41" s="50" t="s">
         <v>350</v>
       </c>
       <c r="K41" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L41" s="50">
         <v>1</v>
@@ -4417,8 +4489,8 @@
       <c r="N41" s="50">
         <v>20</v>
       </c>
-      <c r="O41" s="69" t="s">
-        <v>441</v>
+      <c r="O41" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P41" s="51">
         <v>2.1999999999999999E-2</v>
@@ -4436,54 +4508,54 @@
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="67" t="s">
+      <c r="C42" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="D42" s="72" t="s">
+      <c r="D42" s="61" t="s">
         <v>61</v>
       </c>
-      <c r="E42" s="72" t="s">
+      <c r="E42" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="F42" s="73" t="s">
-        <v>438</v>
-      </c>
-      <c r="G42" s="72" t="s">
+      <c r="F42" s="62" t="s">
+        <v>437</v>
+      </c>
+      <c r="G42" s="61" t="s">
         <v>202</v>
       </c>
-      <c r="H42" s="72" t="s">
-        <v>440</v>
-      </c>
-      <c r="I42" s="72" t="s">
-        <v>440</v>
-      </c>
-      <c r="J42" s="72" t="s">
-        <v>440</v>
-      </c>
-      <c r="K42" s="72" t="s">
-        <v>440</v>
-      </c>
-      <c r="L42" s="72">
+      <c r="H42" s="61" t="s">
+        <v>439</v>
+      </c>
+      <c r="I42" s="61" t="s">
+        <v>439</v>
+      </c>
+      <c r="J42" s="61" t="s">
+        <v>439</v>
+      </c>
+      <c r="K42" s="61" t="s">
+        <v>439</v>
+      </c>
+      <c r="L42" s="61">
         <v>27</v>
       </c>
-      <c r="M42" s="72">
+      <c r="M42" s="61">
         <f>L42*5</f>
         <v>135</v>
       </c>
-      <c r="N42" s="72" t="s">
-        <v>440</v>
-      </c>
-      <c r="O42" s="72" t="s">
-        <v>441</v>
-      </c>
-      <c r="P42" s="74" t="s">
-        <v>440</v>
-      </c>
-      <c r="Q42" s="74" t="s">
-        <v>440</v>
-      </c>
-      <c r="R42" s="72"/>
-      <c r="S42" s="75"/>
+      <c r="N42" s="61" t="s">
+        <v>439</v>
+      </c>
+      <c r="O42" s="61" t="s">
+        <v>440</v>
+      </c>
+      <c r="P42" s="63" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q42" s="63" t="s">
+        <v>439</v>
+      </c>
+      <c r="R42" s="61"/>
+      <c r="S42" s="64"/>
     </row>
     <row r="43" spans="1:19">
       <c r="A43" s="1"/>
@@ -4491,7 +4563,7 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="68" t="s">
+      <c r="C43" s="58" t="s">
         <v>21</v>
       </c>
       <c r="D43" s="50" t="s">
@@ -4510,13 +4582,13 @@
         <v>305</v>
       </c>
       <c r="I43" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J43" s="50" t="s">
         <v>351</v>
       </c>
       <c r="K43" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L43" s="50">
         <v>2</v>
@@ -4528,8 +4600,8 @@
       <c r="N43" s="50">
         <v>11</v>
       </c>
-      <c r="O43" s="69" t="s">
-        <v>441</v>
+      <c r="O43" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P43" s="51">
         <v>1.0055000000000001</v>
@@ -4547,7 +4619,7 @@
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
-      <c r="C44" s="68" t="s">
+      <c r="C44" s="58" t="s">
         <v>21</v>
       </c>
       <c r="D44" s="36" t="s">
@@ -4565,12 +4637,14 @@
       <c r="H44" s="36" t="s">
         <v>306</v>
       </c>
-      <c r="I44" s="36"/>
+      <c r="I44" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J44" s="36" t="s">
         <v>352</v>
       </c>
       <c r="K44" s="36" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L44" s="36">
         <v>1</v>
@@ -4582,8 +4656,8 @@
       <c r="N44" s="36">
         <v>20</v>
       </c>
-      <c r="O44" s="69" t="s">
-        <v>441</v>
+      <c r="O44" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P44" s="37">
         <v>1.9300000000000001E-2</v>
@@ -4601,7 +4675,7 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="68" t="s">
+      <c r="C45" s="58" t="s">
         <v>21</v>
       </c>
       <c r="D45" s="50" t="s">
@@ -4619,12 +4693,14 @@
       <c r="H45" s="50" t="s">
         <v>295</v>
       </c>
-      <c r="I45" s="50"/>
+      <c r="I45" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J45" s="50" t="s">
         <v>353</v>
       </c>
       <c r="K45" s="50" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L45" s="50">
         <v>2</v>
@@ -4636,8 +4712,8 @@
       <c r="N45" s="50">
         <v>20</v>
       </c>
-      <c r="O45" s="69" t="s">
-        <v>441</v>
+      <c r="O45" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P45" s="51">
         <v>1.9099999999999999E-2</v>
@@ -4655,7 +4731,7 @@
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="67" t="s">
+      <c r="C46" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D46" s="36" t="s">
@@ -4673,12 +4749,14 @@
       <c r="H46" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I46" s="36"/>
+      <c r="I46" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J46" s="36" t="s">
         <v>354</v>
       </c>
       <c r="K46" s="36" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="L46" s="36">
         <v>12</v>
@@ -4690,8 +4768,8 @@
       <c r="N46" s="36">
         <v>100</v>
       </c>
-      <c r="O46" s="69" t="s">
-        <v>441</v>
+      <c r="O46" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P46" s="37">
         <v>5.9999999999999995E-4</v>
@@ -4709,7 +4787,7 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="68" t="s">
+      <c r="C47" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D47" s="50" t="s">
@@ -4727,12 +4805,14 @@
       <c r="H47" s="50" t="s">
         <v>307</v>
       </c>
-      <c r="I47" s="50"/>
+      <c r="I47" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J47" s="50" t="s">
         <v>355</v>
       </c>
       <c r="K47" s="50" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L47" s="50">
         <v>1</v>
@@ -4744,8 +4824,8 @@
       <c r="N47" s="50">
         <v>10</v>
       </c>
-      <c r="O47" s="69" t="s">
-        <v>441</v>
+      <c r="O47" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P47" s="51">
         <v>4.1500000000000002E-2</v>
@@ -4763,7 +4843,7 @@
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
-      <c r="C48" s="67" t="s">
+      <c r="C48" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D48" s="36" t="s">
@@ -4781,12 +4861,14 @@
       <c r="H48" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I48" s="36"/>
+      <c r="I48" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J48" s="36" t="s">
         <v>356</v>
       </c>
       <c r="K48" s="36" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="L48" s="36">
         <v>25</v>
@@ -4798,8 +4880,8 @@
       <c r="N48" s="36">
         <v>200</v>
       </c>
-      <c r="O48" s="69" t="s">
-        <v>441</v>
+      <c r="O48" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P48" s="37">
         <v>5.9999999999999995E-4</v>
@@ -4817,7 +4899,7 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C49" s="67" t="s">
+      <c r="C49" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D49" s="50" t="s">
@@ -4835,12 +4917,14 @@
       <c r="H49" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I49" s="50"/>
+      <c r="I49" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J49" s="50" t="s">
         <v>357</v>
       </c>
       <c r="K49" s="50" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L49" s="50">
         <v>2</v>
@@ -4852,8 +4936,8 @@
       <c r="N49" s="50">
         <v>100</v>
       </c>
-      <c r="O49" s="69" t="s">
-        <v>441</v>
+      <c r="O49" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P49" s="51">
         <v>6.9999999999999999E-4</v>
@@ -4871,7 +4955,7 @@
         <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
-      <c r="C50" s="67" t="s">
+      <c r="C50" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D50" s="36" t="s">
@@ -4889,12 +4973,14 @@
       <c r="H50" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I50" s="36"/>
+      <c r="I50" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J50" s="36" t="s">
         <v>358</v>
       </c>
       <c r="K50" s="36" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="L50" s="36">
         <v>3</v>
@@ -4906,8 +4992,8 @@
       <c r="N50" s="36">
         <v>20</v>
       </c>
-      <c r="O50" s="69" t="s">
-        <v>441</v>
+      <c r="O50" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P50" s="37">
         <v>2.4899999999999999E-2</v>
@@ -4925,7 +5011,7 @@
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="68" t="s">
+      <c r="C51" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D51" s="50" t="s">
@@ -4943,12 +5029,14 @@
       <c r="H51" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I51" s="50"/>
+      <c r="I51" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J51" s="50" t="s">
         <v>359</v>
       </c>
       <c r="K51" s="50" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="L51" s="50">
         <v>3</v>
@@ -4960,8 +5048,8 @@
       <c r="N51" s="50">
         <v>20</v>
       </c>
-      <c r="O51" s="69" t="s">
-        <v>441</v>
+      <c r="O51" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P51" s="51">
         <v>1.9E-2</v>
@@ -4979,7 +5067,7 @@
         <f>ROW(B52) - ROW($B$9)</f>
         <v>43</v>
       </c>
-      <c r="C52" s="67" t="s">
+      <c r="C52" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D52" s="36" t="s">
@@ -4997,12 +5085,14 @@
       <c r="H52" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I52" s="36"/>
+      <c r="I52" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J52" s="36" t="s">
         <v>360</v>
       </c>
       <c r="K52" s="36" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="L52" s="36">
         <v>5</v>
@@ -5014,8 +5104,8 @@
       <c r="N52" s="36">
         <v>100</v>
       </c>
-      <c r="O52" s="69" t="s">
-        <v>441</v>
+      <c r="O52" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P52" s="37">
         <v>6.9999999999999999E-4</v>
@@ -5033,7 +5123,7 @@
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C53" s="68" t="s">
+      <c r="C53" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D53" s="50" t="s">
@@ -5045,18 +5135,20 @@
       <c r="F53" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="G53" s="73" t="s">
+      <c r="G53" s="62" t="s">
         <v>258</v>
       </c>
       <c r="H53" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I53" s="50"/>
+      <c r="I53" s="50" t="s">
+        <v>451</v>
+      </c>
       <c r="J53" s="50" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="K53" s="50" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L53" s="50">
         <v>4</v>
@@ -5068,8 +5160,8 @@
       <c r="N53" s="50">
         <v>100</v>
       </c>
-      <c r="O53" s="69" t="s">
-        <v>441</v>
+      <c r="O53" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P53" s="51">
         <v>1.6999999999999999E-3</v>
@@ -5087,7 +5179,7 @@
         <f>ROW(B54) - ROW($B$9)</f>
         <v>45</v>
       </c>
-      <c r="C54" s="67" t="s">
+      <c r="C54" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D54" s="36" t="s">
@@ -5105,12 +5197,14 @@
       <c r="H54" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I54" s="36"/>
+      <c r="I54" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J54" s="36" t="s">
         <v>361</v>
       </c>
       <c r="K54" s="36" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="L54" s="36">
         <v>2</v>
@@ -5122,8 +5216,8 @@
       <c r="N54" s="36">
         <v>100</v>
       </c>
-      <c r="O54" s="69" t="s">
-        <v>441</v>
+      <c r="O54" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P54" s="37">
         <v>6.9999999999999999E-4</v>
@@ -5141,7 +5235,7 @@
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C55" s="68" t="s">
+      <c r="C55" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D55" s="50" t="s">
@@ -5159,12 +5253,14 @@
       <c r="H55" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I55" s="50"/>
+      <c r="I55" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J55" s="50" t="s">
         <v>362</v>
       </c>
       <c r="K55" s="50" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="L55" s="50">
         <v>1</v>
@@ -5176,8 +5272,8 @@
       <c r="N55" s="50">
         <v>100</v>
       </c>
-      <c r="O55" s="69" t="s">
-        <v>441</v>
+      <c r="O55" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P55" s="51">
         <v>1.1999999999999999E-3</v>
@@ -5195,7 +5291,7 @@
         <f>ROW(B56) - ROW($B$9)</f>
         <v>47</v>
       </c>
-      <c r="C56" s="67" t="s">
+      <c r="C56" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D56" s="36" t="s">
@@ -5213,12 +5309,14 @@
       <c r="H56" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I56" s="36"/>
+      <c r="I56" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J56" s="36" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="K56" s="36" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="L56" s="36">
         <v>1</v>
@@ -5230,8 +5328,8 @@
       <c r="N56" s="36">
         <v>20</v>
       </c>
-      <c r="O56" s="69" t="s">
-        <v>441</v>
+      <c r="O56" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P56" s="37">
         <v>3.2399999999999998E-2</v>
@@ -5249,7 +5347,7 @@
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="C57" s="68" t="s">
+      <c r="C57" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D57" s="50" t="s">
@@ -5267,12 +5365,14 @@
       <c r="H57" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I57" s="50"/>
+      <c r="I57" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J57" s="50" t="s">
         <v>363</v>
       </c>
       <c r="K57" s="50" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="L57" s="50">
         <v>1</v>
@@ -5284,8 +5384,8 @@
       <c r="N57" s="50">
         <v>100</v>
       </c>
-      <c r="O57" s="69" t="s">
-        <v>441</v>
+      <c r="O57" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P57" s="51">
         <v>2.2000000000000001E-3</v>
@@ -5303,7 +5403,7 @@
         <f>ROW(B58) - ROW($B$9)</f>
         <v>49</v>
       </c>
-      <c r="C58" s="67" t="s">
+      <c r="C58" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D58" s="36" t="s">
@@ -5321,12 +5421,14 @@
       <c r="H58" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I58" s="36"/>
+      <c r="I58" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J58" s="36" t="s">
         <v>364</v>
       </c>
       <c r="K58" s="36" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L58" s="36">
         <v>31</v>
@@ -5338,8 +5440,8 @@
       <c r="N58" s="36">
         <v>200</v>
       </c>
-      <c r="O58" s="69" t="s">
-        <v>441</v>
+      <c r="O58" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P58" s="37">
         <v>8.0000000000000004E-4</v>
@@ -5357,7 +5459,7 @@
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="C59" s="68" t="s">
+      <c r="C59" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D59" s="50" t="s">
@@ -5375,12 +5477,14 @@
       <c r="H59" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I59" s="50"/>
+      <c r="I59" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J59" s="50" t="s">
         <v>365</v>
       </c>
       <c r="K59" s="50" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L59" s="50">
         <v>5</v>
@@ -5392,8 +5496,8 @@
       <c r="N59" s="50">
         <v>100</v>
       </c>
-      <c r="O59" s="69" t="s">
-        <v>441</v>
+      <c r="O59" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P59" s="51">
         <v>1.1000000000000001E-3</v>
@@ -5411,7 +5515,7 @@
         <f>ROW(B60) - ROW($B$9)</f>
         <v>51</v>
       </c>
-      <c r="C60" s="67" t="s">
+      <c r="C60" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D60" s="36" t="s">
@@ -5429,12 +5533,14 @@
       <c r="H60" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I60" s="36"/>
+      <c r="I60" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J60" s="36" t="s">
         <v>366</v>
       </c>
       <c r="K60" s="36" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L60" s="36">
         <v>36</v>
@@ -5446,8 +5552,8 @@
       <c r="N60" s="36">
         <v>200</v>
       </c>
-      <c r="O60" s="69" t="s">
-        <v>441</v>
+      <c r="O60" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P60" s="37">
         <v>8.9999999999999998E-4</v>
@@ -5465,7 +5571,7 @@
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="C61" s="68" t="s">
+      <c r="C61" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D61" s="50" t="s">
@@ -5483,12 +5589,14 @@
       <c r="H61" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I61" s="50"/>
+      <c r="I61" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J61" s="50" t="s">
         <v>367</v>
       </c>
       <c r="K61" s="50" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L61" s="50">
         <v>1</v>
@@ -5500,8 +5608,8 @@
       <c r="N61" s="50">
         <v>100</v>
       </c>
-      <c r="O61" s="69" t="s">
-        <v>441</v>
+      <c r="O61" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P61" s="51">
         <v>8.9999999999999998E-4</v>
@@ -5519,7 +5627,7 @@
         <f>ROW(B62) - ROW($B$9)</f>
         <v>53</v>
       </c>
-      <c r="C62" s="67" t="s">
+      <c r="C62" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D62" s="36" t="s">
@@ -5537,12 +5645,14 @@
       <c r="H62" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I62" s="36"/>
+      <c r="I62" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J62" s="36" t="s">
         <v>368</v>
       </c>
       <c r="K62" s="36" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="L62" s="36">
         <v>2</v>
@@ -5554,8 +5664,8 @@
       <c r="N62" s="36">
         <v>100</v>
       </c>
-      <c r="O62" s="69" t="s">
-        <v>441</v>
+      <c r="O62" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P62" s="37">
         <v>6.9999999999999999E-4</v>
@@ -5573,7 +5683,7 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C63" s="68" t="s">
+      <c r="C63" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D63" s="50" t="s">
@@ -5591,12 +5701,14 @@
       <c r="H63" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I63" s="50"/>
+      <c r="I63" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J63" s="50" t="s">
         <v>369</v>
       </c>
       <c r="K63" s="50" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="L63" s="50">
         <v>1</v>
@@ -5608,8 +5720,8 @@
       <c r="N63" s="50">
         <v>100</v>
       </c>
-      <c r="O63" s="69" t="s">
-        <v>441</v>
+      <c r="O63" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P63" s="51">
         <v>1.2999999999999999E-3</v>
@@ -5627,54 +5739,56 @@
         <f>ROW(B64) - ROW($B$9)</f>
         <v>55</v>
       </c>
-      <c r="C64" s="67" t="s">
+      <c r="C64" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="D64" s="76" t="s">
+      <c r="D64" s="65" t="s">
         <v>83</v>
       </c>
-      <c r="E64" s="76" t="s">
+      <c r="E64" s="65" t="s">
         <v>148</v>
       </c>
-      <c r="F64" s="76" t="s">
+      <c r="F64" s="65" t="s">
         <v>205</v>
       </c>
-      <c r="G64" s="76" t="s">
+      <c r="G64" s="65" t="s">
         <v>257</v>
       </c>
-      <c r="H64" s="76" t="s">
+      <c r="H64" s="65" t="s">
         <v>288</v>
       </c>
-      <c r="I64" s="76"/>
-      <c r="J64" s="76" t="s">
+      <c r="I64" s="65" t="s">
+        <v>439</v>
+      </c>
+      <c r="J64" s="65" t="s">
         <v>360</v>
       </c>
-      <c r="K64" s="76" t="s">
-        <v>418</v>
-      </c>
-      <c r="L64" s="76">
+      <c r="K64" s="65" t="s">
+        <v>417</v>
+      </c>
+      <c r="L64" s="65">
         <v>2</v>
       </c>
-      <c r="M64" s="76">
+      <c r="M64" s="65">
         <f>L64*5</f>
         <v>10</v>
       </c>
-      <c r="N64" s="76" t="s">
-        <v>440</v>
-      </c>
-      <c r="O64" s="76" t="s">
-        <v>440</v>
-      </c>
-      <c r="P64" s="77" t="s">
-        <v>440</v>
-      </c>
-      <c r="Q64" s="77" t="s">
-        <v>440</v>
-      </c>
-      <c r="R64" s="79" t="s">
-        <v>443</v>
-      </c>
-      <c r="S64" s="78"/>
+      <c r="N64" s="65" t="s">
+        <v>439</v>
+      </c>
+      <c r="O64" s="65" t="s">
+        <v>439</v>
+      </c>
+      <c r="P64" s="66" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q64" s="66" t="s">
+        <v>439</v>
+      </c>
+      <c r="R64" s="68" t="s">
+        <v>442</v>
+      </c>
+      <c r="S64" s="67"/>
     </row>
     <row r="65" spans="1:19">
       <c r="A65" s="1"/>
@@ -5682,7 +5796,7 @@
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C65" s="68" t="s">
+      <c r="C65" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D65" s="50" t="s">
@@ -5700,12 +5814,14 @@
       <c r="H65" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I65" s="50"/>
+      <c r="I65" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J65" s="50" t="s">
         <v>370</v>
       </c>
       <c r="K65" s="50" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="L65" s="50">
         <v>2</v>
@@ -5717,8 +5833,8 @@
       <c r="N65" s="50">
         <v>100</v>
       </c>
-      <c r="O65" s="69" t="s">
-        <v>441</v>
+      <c r="O65" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P65" s="51">
         <v>2.0999999999999999E-3</v>
@@ -5736,7 +5852,7 @@
         <f>ROW(B66) - ROW($B$9)</f>
         <v>57</v>
       </c>
-      <c r="C66" s="67" t="s">
+      <c r="C66" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D66" s="36" t="s">
@@ -5754,12 +5870,14 @@
       <c r="H66" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I66" s="36"/>
+      <c r="I66" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J66" s="36" t="s">
         <v>371</v>
       </c>
       <c r="K66" s="36" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="L66" s="36">
         <v>1</v>
@@ -5771,8 +5889,8 @@
       <c r="N66" s="36">
         <v>20</v>
       </c>
-      <c r="O66" s="69" t="s">
-        <v>441</v>
+      <c r="O66" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P66" s="37">
         <v>1.9900000000000001E-2</v>
@@ -5790,7 +5908,7 @@
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C67" s="68" t="s">
+      <c r="C67" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D67" s="50" t="s">
@@ -5808,12 +5926,14 @@
       <c r="H67" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I67" s="50"/>
+      <c r="I67" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J67" s="50" t="s">
         <v>372</v>
       </c>
       <c r="K67" s="50" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="L67" s="50">
         <v>1</v>
@@ -5825,8 +5945,8 @@
       <c r="N67" s="50">
         <v>20</v>
       </c>
-      <c r="O67" s="69" t="s">
-        <v>441</v>
+      <c r="O67" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P67" s="51">
         <v>2.53E-2</v>
@@ -5844,7 +5964,7 @@
         <f>ROW(B68) - ROW($B$9)</f>
         <v>59</v>
       </c>
-      <c r="C68" s="67" t="s">
+      <c r="C68" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D68" s="36" t="s">
@@ -5862,12 +5982,14 @@
       <c r="H68" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I68" s="36"/>
+      <c r="I68" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J68" s="36" t="s">
         <v>373</v>
       </c>
       <c r="K68" s="36" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="L68" s="36">
         <v>2</v>
@@ -5879,8 +6001,8 @@
       <c r="N68" s="36">
         <v>20</v>
       </c>
-      <c r="O68" s="69" t="s">
-        <v>441</v>
+      <c r="O68" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P68" s="37">
         <v>3.1E-2</v>
@@ -5898,7 +6020,7 @@
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="C69" s="68" t="s">
+      <c r="C69" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D69" s="50" t="s">
@@ -5916,12 +6038,14 @@
       <c r="H69" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="I69" s="50"/>
+      <c r="I69" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J69" s="50" t="s">
         <v>374</v>
       </c>
       <c r="K69" s="50" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="L69" s="50">
         <v>2</v>
@@ -5933,8 +6057,8 @@
       <c r="N69" s="50">
         <v>20</v>
       </c>
-      <c r="O69" s="69" t="s">
-        <v>441</v>
+      <c r="O69" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P69" s="51">
         <v>2.41E-2</v>
@@ -5952,7 +6076,7 @@
         <f>ROW(B70) - ROW($B$9)</f>
         <v>61</v>
       </c>
-      <c r="C70" s="67" t="s">
+      <c r="C70" s="57" t="s">
         <v>22</v>
       </c>
       <c r="D70" s="36" t="s">
@@ -5970,12 +6094,14 @@
       <c r="H70" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="I70" s="36"/>
+      <c r="I70" s="50" t="s">
+        <v>439</v>
+      </c>
       <c r="J70" s="36" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="K70" s="36" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="L70" s="36">
         <v>2</v>
@@ -5987,8 +6113,8 @@
       <c r="N70" s="36">
         <v>100</v>
       </c>
-      <c r="O70" s="69" t="s">
-        <v>441</v>
+      <c r="O70" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P70" s="37">
         <v>6.9999999999999999E-4</v>
@@ -6006,54 +6132,54 @@
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="C71" s="68" t="s">
+      <c r="C71" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="D71" s="80" t="s">
+      <c r="D71" s="69" t="s">
         <v>90</v>
       </c>
-      <c r="E71" s="80" t="s">
+      <c r="E71" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="F71" s="80" t="s">
-        <v>438</v>
-      </c>
-      <c r="G71" s="80" t="s">
+      <c r="F71" s="69" t="s">
+        <v>437</v>
+      </c>
+      <c r="G71" s="69" t="s">
         <v>211</v>
       </c>
-      <c r="H71" s="80" t="s">
-        <v>440</v>
-      </c>
-      <c r="I71" s="80" t="s">
-        <v>440</v>
-      </c>
-      <c r="J71" s="80" t="s">
-        <v>440</v>
-      </c>
-      <c r="K71" s="80" t="s">
-        <v>440</v>
-      </c>
-      <c r="L71" s="80">
+      <c r="H71" s="69" t="s">
+        <v>439</v>
+      </c>
+      <c r="I71" s="69" t="s">
+        <v>439</v>
+      </c>
+      <c r="J71" s="69" t="s">
+        <v>439</v>
+      </c>
+      <c r="K71" s="69" t="s">
+        <v>439</v>
+      </c>
+      <c r="L71" s="69">
         <v>1</v>
       </c>
-      <c r="M71" s="80">
+      <c r="M71" s="69">
         <f t="shared" ref="M71" si="61">L71*5</f>
         <v>5</v>
       </c>
-      <c r="N71" s="80" t="s">
-        <v>440</v>
-      </c>
-      <c r="O71" s="76" t="s">
-        <v>440</v>
-      </c>
-      <c r="P71" s="81" t="s">
-        <v>440</v>
-      </c>
-      <c r="Q71" s="81" t="s">
-        <v>440</v>
-      </c>
-      <c r="R71" s="79" t="s">
-        <v>443</v>
+      <c r="N71" s="69" t="s">
+        <v>439</v>
+      </c>
+      <c r="O71" s="65" t="s">
+        <v>439</v>
+      </c>
+      <c r="P71" s="70" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q71" s="70" t="s">
+        <v>439</v>
+      </c>
+      <c r="R71" s="68" t="s">
+        <v>442</v>
       </c>
       <c r="S71" s="55"/>
     </row>
@@ -6063,7 +6189,7 @@
         <f>ROW(B72) - ROW($B$9)</f>
         <v>63</v>
       </c>
-      <c r="C72" s="67" t="s">
+      <c r="C72" s="57" t="s">
         <v>24</v>
       </c>
       <c r="D72" s="36" t="s">
@@ -6073,7 +6199,7 @@
         <v>167</v>
       </c>
       <c r="F72" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G72" s="36" t="s">
         <v>212</v>
@@ -6081,11 +6207,15 @@
       <c r="H72" s="36" t="s">
         <v>300</v>
       </c>
-      <c r="I72" s="36"/>
+      <c r="I72" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J72" s="36" t="s">
         <v>375</v>
       </c>
-      <c r="K72" s="36"/>
+      <c r="K72" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L72" s="36">
         <v>2</v>
       </c>
@@ -6096,8 +6226,8 @@
       <c r="N72" s="36">
         <v>20</v>
       </c>
-      <c r="O72" s="69" t="s">
-        <v>441</v>
+      <c r="O72" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P72" s="37">
         <v>2.1700000000000001E-2</v>
@@ -6115,7 +6245,7 @@
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="C73" s="68" t="s">
+      <c r="C73" s="58" t="s">
         <v>25</v>
       </c>
       <c r="D73" s="50" t="s">
@@ -6133,11 +6263,15 @@
       <c r="H73" s="50" t="s">
         <v>308</v>
       </c>
-      <c r="I73" s="50"/>
+      <c r="I73" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J73" s="50" t="s">
         <v>376</v>
       </c>
-      <c r="K73" s="50"/>
+      <c r="K73" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L73" s="50">
         <v>1</v>
       </c>
@@ -6148,8 +6282,8 @@
       <c r="N73" s="50">
         <v>6</v>
       </c>
-      <c r="O73" s="69" t="s">
-        <v>441</v>
+      <c r="O73" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P73" s="51">
         <v>2.2766999999999999</v>
@@ -6167,7 +6301,7 @@
         <f>ROW(B74) - ROW($B$9)</f>
         <v>65</v>
       </c>
-      <c r="C74" s="67" t="s">
+      <c r="C74" s="57" t="s">
         <v>25</v>
       </c>
       <c r="D74" s="36" t="s">
@@ -6185,11 +6319,15 @@
       <c r="H74" s="36" t="s">
         <v>309</v>
       </c>
-      <c r="I74" s="36"/>
+      <c r="I74" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J74" s="36" t="s">
         <v>377</v>
       </c>
-      <c r="K74" s="36"/>
+      <c r="K74" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L74" s="36">
         <v>1</v>
       </c>
@@ -6200,8 +6338,8 @@
       <c r="N74" s="36">
         <v>6</v>
       </c>
-      <c r="O74" s="69" t="s">
-        <v>441</v>
+      <c r="O74" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P74" s="37">
         <v>1.2537</v>
@@ -6219,7 +6357,7 @@
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="C75" s="68" t="s">
+      <c r="C75" s="58" t="s">
         <v>25</v>
       </c>
       <c r="D75" s="50" t="s">
@@ -6237,11 +6375,15 @@
       <c r="H75" s="50" t="s">
         <v>308</v>
       </c>
-      <c r="I75" s="50"/>
+      <c r="I75" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J75" s="50" t="s">
         <v>378</v>
       </c>
-      <c r="K75" s="50"/>
+      <c r="K75" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L75" s="50">
         <v>4</v>
       </c>
@@ -6252,8 +6394,8 @@
       <c r="N75" s="50">
         <v>21</v>
       </c>
-      <c r="O75" s="69" t="s">
-        <v>441</v>
+      <c r="O75" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P75" s="51">
         <v>0.72550000000000003</v>
@@ -6271,7 +6413,7 @@
         <f>ROW(B76) - ROW($B$9)</f>
         <v>67</v>
       </c>
-      <c r="C76" s="67" t="s">
+      <c r="C76" s="57" t="s">
         <v>25</v>
       </c>
       <c r="D76" s="36" t="s">
@@ -6289,11 +6431,15 @@
       <c r="H76" s="36" t="s">
         <v>310</v>
       </c>
-      <c r="I76" s="36"/>
+      <c r="I76" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J76" s="36" t="s">
         <v>379</v>
       </c>
-      <c r="K76" s="36"/>
+      <c r="K76" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L76" s="36">
         <v>1</v>
       </c>
@@ -6304,8 +6450,8 @@
       <c r="N76" s="36">
         <v>10</v>
       </c>
-      <c r="O76" s="69" t="s">
-        <v>441</v>
+      <c r="O76" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P76" s="37">
         <v>0.32879999999999998</v>
@@ -6323,7 +6469,7 @@
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
-      <c r="C77" s="68" t="s">
+      <c r="C77" s="58" t="s">
         <v>25</v>
       </c>
       <c r="D77" s="50" t="s">
@@ -6341,11 +6487,15 @@
       <c r="H77" s="50" t="s">
         <v>311</v>
       </c>
-      <c r="I77" s="50"/>
+      <c r="I77" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J77" s="50" t="s">
         <v>380</v>
       </c>
-      <c r="K77" s="50"/>
+      <c r="K77" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L77" s="50">
         <v>1</v>
       </c>
@@ -6356,8 +6506,8 @@
       <c r="N77" s="50">
         <v>10</v>
       </c>
-      <c r="O77" s="69" t="s">
-        <v>441</v>
+      <c r="O77" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P77" s="51">
         <v>0.33800000000000002</v>
@@ -6375,7 +6525,7 @@
         <f>ROW(B78) - ROW($B$9)</f>
         <v>69</v>
       </c>
-      <c r="C78" s="67" t="s">
+      <c r="C78" s="57" t="s">
         <v>26</v>
       </c>
       <c r="D78" s="36" t="s">
@@ -6393,11 +6543,15 @@
       <c r="H78" s="36" t="s">
         <v>312</v>
       </c>
-      <c r="I78" s="36"/>
+      <c r="I78" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J78" s="36" t="s">
         <v>381</v>
       </c>
-      <c r="K78" s="36"/>
+      <c r="K78" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L78" s="36">
         <v>1</v>
       </c>
@@ -6408,8 +6562,8 @@
       <c r="N78" s="36">
         <v>6</v>
       </c>
-      <c r="O78" s="69" t="s">
-        <v>441</v>
+      <c r="O78" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P78" s="37">
         <v>5.1721000000000004</v>
@@ -6427,7 +6581,7 @@
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="C79" s="68" t="s">
+      <c r="C79" s="58" t="s">
         <v>25</v>
       </c>
       <c r="D79" s="50" t="s">
@@ -6445,11 +6599,15 @@
       <c r="H79" s="50" t="s">
         <v>313</v>
       </c>
-      <c r="I79" s="50"/>
+      <c r="I79" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J79" s="50" t="s">
         <v>382</v>
       </c>
-      <c r="K79" s="50"/>
+      <c r="K79" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L79" s="50">
         <v>1</v>
       </c>
@@ -6460,8 +6618,8 @@
       <c r="N79" s="50">
         <v>6</v>
       </c>
-      <c r="O79" s="69" t="s">
-        <v>441</v>
+      <c r="O79" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P79" s="51">
         <v>16.753900000000002</v>
@@ -6479,7 +6637,7 @@
         <f>ROW(B80) - ROW($B$9)</f>
         <v>71</v>
       </c>
-      <c r="C80" s="67" t="s">
+      <c r="C80" s="57" t="s">
         <v>25</v>
       </c>
       <c r="D80" s="36" t="s">
@@ -6497,11 +6655,15 @@
       <c r="H80" s="36" t="s">
         <v>314</v>
       </c>
-      <c r="I80" s="36"/>
+      <c r="I80" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J80" s="36" t="s">
         <v>383</v>
       </c>
-      <c r="K80" s="36"/>
+      <c r="K80" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L80" s="36">
         <v>1</v>
       </c>
@@ -6512,8 +6674,8 @@
       <c r="N80" s="36">
         <v>10</v>
       </c>
-      <c r="O80" s="69" t="s">
-        <v>441</v>
+      <c r="O80" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P80" s="37">
         <v>0.30580000000000002</v>
@@ -6531,7 +6693,7 @@
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="C81" s="68" t="s">
+      <c r="C81" s="58" t="s">
         <v>25</v>
       </c>
       <c r="D81" s="50" t="s">
@@ -6549,11 +6711,15 @@
       <c r="H81" s="50" t="s">
         <v>315</v>
       </c>
-      <c r="I81" s="50"/>
+      <c r="I81" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J81" s="50" t="s">
         <v>384</v>
       </c>
-      <c r="K81" s="50"/>
+      <c r="K81" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L81" s="50">
         <v>2</v>
       </c>
@@ -6564,8 +6730,8 @@
       <c r="N81" s="50">
         <v>15</v>
       </c>
-      <c r="O81" s="69" t="s">
-        <v>441</v>
+      <c r="O81" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P81" s="51">
         <v>0.34520000000000001</v>
@@ -6583,7 +6749,7 @@
         <f>ROW(B82) - ROW($B$9)</f>
         <v>73</v>
       </c>
-      <c r="C82" s="67" t="s">
+      <c r="C82" s="57" t="s">
         <v>27</v>
       </c>
       <c r="D82" s="36" t="s">
@@ -6593,7 +6759,7 @@
         <v>177</v>
       </c>
       <c r="F82" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G82" s="36" t="s">
         <v>219</v>
@@ -6601,11 +6767,15 @@
       <c r="H82" s="36" t="s">
         <v>316</v>
       </c>
-      <c r="I82" s="36"/>
+      <c r="I82" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J82" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="K82" s="36"/>
+      <c r="K82" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L82" s="36">
         <v>3</v>
       </c>
@@ -6616,8 +6786,8 @@
       <c r="N82" s="36">
         <v>16</v>
       </c>
-      <c r="O82" s="69" t="s">
-        <v>441</v>
+      <c r="O82" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P82" s="37">
         <v>1.7230000000000001</v>
@@ -6635,7 +6805,7 @@
         <f t="shared" si="0"/>
         <v>74</v>
       </c>
-      <c r="C83" s="68" t="s">
+      <c r="C83" s="58" t="s">
         <v>25</v>
       </c>
       <c r="D83" s="50" t="s">
@@ -6653,11 +6823,15 @@
       <c r="H83" s="50" t="s">
         <v>308</v>
       </c>
-      <c r="I83" s="50"/>
+      <c r="I83" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J83" s="50" t="s">
         <v>386</v>
       </c>
-      <c r="K83" s="50"/>
+      <c r="K83" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L83" s="50">
         <v>1</v>
       </c>
@@ -6668,8 +6842,8 @@
       <c r="N83" s="50">
         <v>6</v>
       </c>
-      <c r="O83" s="69" t="s">
-        <v>441</v>
+      <c r="O83" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P83" s="51">
         <v>1.0660000000000001</v>
@@ -6681,13 +6855,13 @@
       <c r="R83" s="50"/>
       <c r="S83" s="55"/>
     </row>
-    <row r="84" spans="1:19">
-      <c r="A84" s="1"/>
+    <row r="84" spans="1:19" s="82" customFormat="1">
+      <c r="A84" s="81"/>
       <c r="B84" s="45">
         <f>ROW(B84) - ROW($B$9)</f>
         <v>75</v>
       </c>
-      <c r="C84" s="67" t="s">
+      <c r="C84" s="57" t="s">
         <v>25</v>
       </c>
       <c r="D84" s="36" t="s">
@@ -6705,11 +6879,15 @@
       <c r="H84" s="36" t="s">
         <v>317</v>
       </c>
-      <c r="I84" s="36"/>
+      <c r="I84" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J84" s="36" t="s">
-        <v>387</v>
-      </c>
-      <c r="K84" s="36"/>
+        <v>439</v>
+      </c>
+      <c r="K84" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="L84" s="36">
         <v>1</v>
       </c>
@@ -6717,23 +6895,29 @@
         <f>L84*5</f>
         <v>5</v>
       </c>
-      <c r="N84" s="36"/>
-      <c r="O84" s="36"/>
-      <c r="P84" s="37"/>
+      <c r="N84" s="36">
+        <v>6</v>
+      </c>
+      <c r="O84" s="59" t="s">
+        <v>450</v>
+      </c>
+      <c r="P84" s="37">
+        <v>2.7029999999999998</v>
+      </c>
       <c r="Q84" s="37">
         <f>P84*N84</f>
-        <v>0</v>
+        <v>16.218</v>
       </c>
       <c r="R84" s="36"/>
       <c r="S84" s="55"/>
     </row>
-    <row r="85" spans="1:19" ht="24.75" thickBot="1">
-      <c r="A85" s="1"/>
+    <row r="85" spans="1:19" s="82" customFormat="1" ht="24.75" thickBot="1">
+      <c r="A85" s="81"/>
       <c r="B85" s="46">
         <f t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="C85" s="68" t="s">
+      <c r="C85" s="58" t="s">
         <v>28</v>
       </c>
       <c r="D85" s="50" t="s">
@@ -6743,7 +6927,7 @@
         <v>180</v>
       </c>
       <c r="F85" s="50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G85" s="50" t="s">
         <v>286</v>
@@ -6751,95 +6935,181 @@
       <c r="H85" s="50" t="s">
         <v>318</v>
       </c>
-      <c r="I85" s="50"/>
+      <c r="I85" s="36" t="s">
+        <v>439</v>
+      </c>
       <c r="J85" s="50" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="K85" s="50" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="L85" s="50">
         <v>1</v>
       </c>
       <c r="M85" s="50">
-        <f t="shared" ref="M85" si="74">L85*5</f>
+        <f t="shared" ref="M85:M86" si="74">L85*5</f>
         <v>5</v>
       </c>
       <c r="N85" s="50">
         <v>6</v>
       </c>
-      <c r="O85" s="69" t="s">
-        <v>441</v>
+      <c r="O85" s="59" t="s">
+        <v>440</v>
       </c>
       <c r="P85" s="51">
         <v>0.1152</v>
       </c>
       <c r="Q85" s="51">
-        <f t="shared" ref="Q85" si="75">P85*N85</f>
+        <f t="shared" ref="Q85:Q86" si="75">P85*N85</f>
         <v>0.69120000000000004</v>
       </c>
       <c r="R85" s="50"/>
       <c r="S85" s="38"/>
     </row>
-    <row r="86" spans="1:19" ht="19.5" thickBot="1">
-      <c r="A86" s="1"/>
-      <c r="B86" s="39"/>
-      <c r="C86" s="40"/>
-      <c r="D86" s="41"/>
-      <c r="E86" s="42"/>
-      <c r="F86" s="43"/>
-      <c r="G86" s="44"/>
-      <c r="H86" s="43"/>
-      <c r="I86" s="44"/>
-      <c r="J86" s="43"/>
-      <c r="K86" s="44"/>
-      <c r="L86" s="44"/>
-      <c r="M86" s="44"/>
-      <c r="N86" s="64" t="s">
+    <row r="86" spans="1:19" s="82" customFormat="1" ht="24.75" thickBot="1">
+      <c r="A86" s="81"/>
+      <c r="B86" s="46">
+        <f t="shared" si="0"/>
+        <v>77</v>
+      </c>
+      <c r="C86" s="58" t="s">
+        <v>445</v>
+      </c>
+      <c r="D86" s="50" t="s">
+        <v>439</v>
+      </c>
+      <c r="E86" s="50" t="s">
+        <v>447</v>
+      </c>
+      <c r="F86" s="50" t="s">
+        <v>439</v>
+      </c>
+      <c r="G86" s="50" t="s">
+        <v>446</v>
+      </c>
+      <c r="H86" s="50" t="s">
+        <v>439</v>
+      </c>
+      <c r="I86" s="50" t="s">
+        <v>439</v>
+      </c>
+      <c r="J86" s="50" t="s">
+        <v>439</v>
+      </c>
+      <c r="K86" s="50" t="s">
+        <v>439</v>
+      </c>
+      <c r="L86" s="50">
+        <v>1</v>
+      </c>
+      <c r="M86" s="50">
+        <f t="shared" si="74"/>
         <v>5</v>
       </c>
-      <c r="O86" s="65"/>
-      <c r="P86" s="65"/>
-      <c r="Q86" s="47">
-        <f>SUM(Q10:Q85)</f>
-        <v>301.16679999999991</v>
-      </c>
-      <c r="R86" s="60"/>
-      <c r="S86" s="61"/>
-    </row>
-    <row r="87" spans="1:19" ht="19.5" thickBot="1">
+      <c r="N86" s="50">
+        <v>6</v>
+      </c>
+      <c r="O86" s="59" t="s">
+        <v>449</v>
+      </c>
+      <c r="P86" s="51">
+        <v>12.09</v>
+      </c>
+      <c r="Q86" s="51">
+        <f t="shared" si="75"/>
+        <v>72.539999999999992</v>
+      </c>
+      <c r="R86" s="50"/>
+      <c r="S86" s="38"/>
+    </row>
+    <row r="87" spans="1:19" ht="15.75" thickBot="1">
       <c r="A87" s="1"/>
-      <c r="B87" s="25"/>
-      <c r="C87" s="35"/>
-      <c r="D87" s="9"/>
-      <c r="E87" s="10"/>
-      <c r="F87" s="10"/>
-      <c r="G87" s="10"/>
-      <c r="H87" s="10"/>
-      <c r="I87" s="10"/>
-      <c r="J87" s="10"/>
-      <c r="K87" s="10"/>
-      <c r="L87" s="10"/>
-      <c r="M87" s="10"/>
-      <c r="N87" s="64" t="s">
+      <c r="B87" s="46">
+        <f t="shared" ref="B87" si="76">ROW(B87) - ROW($B$9)</f>
+        <v>78</v>
+      </c>
+      <c r="C87" s="58" t="s">
+        <v>445</v>
+      </c>
+      <c r="D87" s="50"/>
+      <c r="E87" s="50"/>
+      <c r="F87" s="50"/>
+      <c r="G87" s="50" t="s">
+        <v>448</v>
+      </c>
+      <c r="H87" s="50"/>
+      <c r="I87" s="50"/>
+      <c r="J87" s="50"/>
+      <c r="K87" s="50"/>
+      <c r="L87" s="50"/>
+      <c r="M87" s="50"/>
+      <c r="N87" s="50"/>
+      <c r="O87" s="59"/>
+      <c r="P87" s="51"/>
+      <c r="Q87" s="51"/>
+      <c r="R87" s="50"/>
+      <c r="S87" s="38"/>
+    </row>
+    <row r="88" spans="1:19" ht="19.5" thickBot="1">
+      <c r="A88" s="1"/>
+      <c r="B88" s="39"/>
+      <c r="C88" s="40"/>
+      <c r="D88" s="41"/>
+      <c r="E88" s="42"/>
+      <c r="F88" s="43"/>
+      <c r="G88" s="44"/>
+      <c r="H88" s="43"/>
+      <c r="I88" s="44"/>
+      <c r="J88" s="43"/>
+      <c r="K88" s="44"/>
+      <c r="L88" s="44"/>
+      <c r="M88" s="44"/>
+      <c r="N88" s="79" t="s">
+        <v>5</v>
+      </c>
+      <c r="O88" s="80"/>
+      <c r="P88" s="80"/>
+      <c r="Q88" s="47">
+        <f>SUM(Q10:Q87)</f>
+        <v>390.0447999999999</v>
+      </c>
+      <c r="R88" s="75"/>
+      <c r="S88" s="76"/>
+    </row>
+    <row r="89" spans="1:19" ht="19.5" thickBot="1">
+      <c r="A89" s="1"/>
+      <c r="B89" s="25"/>
+      <c r="C89" s="35"/>
+      <c r="D89" s="9"/>
+      <c r="E89" s="10"/>
+      <c r="F89" s="10"/>
+      <c r="G89" s="10"/>
+      <c r="H89" s="10"/>
+      <c r="I89" s="10"/>
+      <c r="J89" s="10"/>
+      <c r="K89" s="10"/>
+      <c r="L89" s="10"/>
+      <c r="M89" s="10"/>
+      <c r="N89" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="O87" s="65"/>
-      <c r="P87" s="65"/>
-      <c r="Q87" s="48">
-        <f>Q86/5</f>
-        <v>60.233359999999983</v>
-      </c>
-      <c r="R87" s="62"/>
-      <c r="S87" s="63"/>
+      <c r="O89" s="80"/>
+      <c r="P89" s="80"/>
+      <c r="Q89" s="48">
+        <f>Q88/5</f>
+        <v>78.008959999999973</v>
+      </c>
+      <c r="R89" s="77"/>
+      <c r="S89" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="R86:S87"/>
-    <mergeCell ref="N86:P86"/>
-    <mergeCell ref="N87:P87"/>
+    <mergeCell ref="R88:S89"/>
+    <mergeCell ref="N88:P88"/>
+    <mergeCell ref="N89:P89"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O10" r:id="rId1"/>
@@ -6914,9 +7184,11 @@
     <hyperlink ref="O83" r:id="rId70"/>
     <hyperlink ref="O85" r:id="rId71"/>
     <hyperlink ref="O53" r:id="rId72"/>
+    <hyperlink ref="O86" r:id="rId73"/>
+    <hyperlink ref="O84" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId73"/>
-  <drawing r:id="rId74"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId75"/>
+  <drawing r:id="rId76"/>
 </worksheet>
 </file>
</xml_diff>